<commit_message>
add all information from index
</commit_message>
<xml_diff>
--- a/data/stories_index.xlsx
+++ b/data/stories_index.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="761" uniqueCount="310">
   <si>
     <t>Number</t>
   </si>
@@ -71,6 +71,9 @@
   </si>
   <si>
     <t>Check Lenneke?</t>
+  </si>
+  <si>
+    <t>Lenneke's rating (e.g. is the text "good" --&gt; interesting/informative and well written). 1 = very bad, 5 = very good</t>
   </si>
   <si>
     <t>“Mijn Heer Zak met Rijst”</t>
@@ -1474,38 +1477,41 @@
       <c r="U1" s="10" t="s">
         <v>19</v>
       </c>
+      <c r="V1" s="10" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="10">
         <v>1.0</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C2" s="11"/>
       <c r="D2" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F2" s="10">
         <v>826.0</v>
       </c>
       <c r="G2" s="12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I2" s="13">
         <v>45205.0</v>
       </c>
       <c r="J2" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K2" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L2" s="10">
         <v>0.0</v>
@@ -1527,10 +1533,10 @@
       </c>
       <c r="S2" s="9"/>
       <c r="T2" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U2" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3">
@@ -1538,32 +1544,32 @@
         <v>2.0</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C3" s="16"/>
       <c r="D3" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F3" s="10">
         <v>801.0</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I3" s="13">
         <v>45205.0</v>
       </c>
       <c r="J3" s="17" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="K3" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L3" s="10">
         <v>0.0</v>
@@ -1585,10 +1591,10 @@
       </c>
       <c r="S3" s="18"/>
       <c r="T3" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U3" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4">
@@ -1596,32 +1602,32 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C4" s="20"/>
       <c r="D4" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F4" s="10">
         <v>857.0</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I4" s="13">
         <v>45205.0</v>
       </c>
       <c r="J4" s="17" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L4" s="10">
         <v>0.0</v>
@@ -1643,10 +1649,10 @@
       </c>
       <c r="S4" s="18"/>
       <c r="T4" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U4" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5">
@@ -1654,32 +1660,32 @@
         <v>4.0</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C5" s="21"/>
       <c r="D5" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F5" s="10">
         <v>799.0</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I5" s="13">
         <v>45205.0</v>
       </c>
       <c r="J5" s="17" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L5" s="10">
         <v>0.0</v>
@@ -1701,10 +1707,10 @@
       </c>
       <c r="S5" s="18"/>
       <c r="T5" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
@@ -1712,32 +1718,32 @@
         <v>5.0</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" s="15"/>
       <c r="D6" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F6" s="10">
         <v>797.0</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I6" s="13">
         <v>45205.0</v>
       </c>
       <c r="J6" s="17" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K6" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L6" s="10">
         <v>0.0</v>
@@ -1759,10 +1765,10 @@
       </c>
       <c r="S6" s="18"/>
       <c r="T6" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7">
@@ -1770,32 +1776,32 @@
         <v>6.0</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C7" s="22"/>
       <c r="D7" s="10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F7" s="10">
         <v>893.0</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I7" s="13">
         <v>45205.0</v>
       </c>
       <c r="J7" s="17" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L7" s="10">
         <v>0.0</v>
@@ -1817,10 +1823,10 @@
       </c>
       <c r="S7" s="18"/>
       <c r="T7" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U7" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8">
@@ -1828,32 +1834,32 @@
         <v>7.0</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C8" s="9"/>
       <c r="D8" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F8" s="10">
         <v>891.0</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I8" s="13">
         <v>45205.0</v>
       </c>
       <c r="J8" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="K8" s="10" t="s">
         <v>40</v>
-      </c>
-      <c r="K8" s="10" t="s">
-        <v>39</v>
       </c>
       <c r="L8" s="10">
         <v>0.0</v>
@@ -1875,10 +1881,10 @@
       </c>
       <c r="S8" s="18"/>
       <c r="T8" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U8" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9">
@@ -1886,32 +1892,32 @@
         <v>8.0</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C9" s="9"/>
       <c r="D9" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F9" s="10">
         <v>863.0</v>
       </c>
       <c r="G9" s="23" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H9" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I9" s="13">
         <v>45205.0</v>
       </c>
       <c r="J9" s="17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L9" s="10">
         <v>1.0</v>
@@ -1933,10 +1939,10 @@
       </c>
       <c r="S9" s="18"/>
       <c r="T9" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U9" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10">
@@ -1944,32 +1950,32 @@
         <v>9.0</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C10" s="9"/>
       <c r="D10" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F10" s="10">
         <v>815.0</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I10" s="13">
         <v>45205.0</v>
       </c>
       <c r="J10" s="17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L10" s="10">
         <v>0.0</v>
@@ -1990,13 +1996,13 @@
         <v>0.0</v>
       </c>
       <c r="S10" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="T10" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U10" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11">
@@ -2004,32 +2010,32 @@
         <v>10.0</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C11" s="9"/>
       <c r="D11" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F11" s="10">
         <v>906.0</v>
       </c>
       <c r="G11" s="12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H11" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I11" s="13">
         <v>45205.0</v>
       </c>
       <c r="J11" s="17" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K11" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L11" s="10">
         <v>0.0</v>
@@ -2051,10 +2057,10 @@
       </c>
       <c r="S11" s="18"/>
       <c r="T11" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U11" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12">
@@ -2062,32 +2068,32 @@
         <v>11.0</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C12" s="9"/>
       <c r="D12" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F12" s="10">
         <v>849.0</v>
       </c>
       <c r="G12" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H12" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I12" s="13">
         <v>45205.0</v>
       </c>
       <c r="J12" s="17" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L12" s="10">
         <v>0.0</v>
@@ -2108,13 +2114,13 @@
         <v>0.0</v>
       </c>
       <c r="S12" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="T12" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U12" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13">
@@ -2122,32 +2128,32 @@
         <v>12.0</v>
       </c>
       <c r="B13" s="24" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C13" s="24"/>
       <c r="D13" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F13" s="10">
         <v>907.0</v>
       </c>
       <c r="G13" s="12" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I13" s="13">
         <v>45205.0</v>
       </c>
       <c r="J13" s="17" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L13" s="10">
         <v>0.0</v>
@@ -2168,13 +2174,13 @@
         <v>0.0</v>
       </c>
       <c r="S13" s="9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="T13" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U13" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14">
@@ -2182,32 +2188,32 @@
         <v>13.0</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C14" s="9"/>
       <c r="D14" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F14" s="10">
         <v>919.0</v>
       </c>
       <c r="G14" s="12" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H14" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I14" s="13">
         <v>45205.0</v>
       </c>
       <c r="J14" s="17" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L14" s="10">
         <v>0.0</v>
@@ -2229,10 +2235,10 @@
       </c>
       <c r="S14" s="18"/>
       <c r="T14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15">
@@ -2240,32 +2246,32 @@
         <v>14.0</v>
       </c>
       <c r="B15" s="25" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C15" s="25"/>
       <c r="D15" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F15" s="10">
         <v>861.0</v>
       </c>
       <c r="G15" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I15" s="13">
         <v>45205.0</v>
       </c>
       <c r="J15" s="17" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L15" s="10">
         <v>2.0</v>
@@ -2286,13 +2292,13 @@
         <v>1.0</v>
       </c>
       <c r="S15" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="T15" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16">
@@ -2300,32 +2306,32 @@
         <v>15.0</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C16" s="9"/>
       <c r="D16" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F16" s="10">
         <v>888.0</v>
       </c>
       <c r="G16" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I16" s="13">
         <v>45205.0</v>
       </c>
       <c r="J16" s="17" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L16" s="10">
         <v>0.0</v>
@@ -2347,10 +2353,10 @@
       </c>
       <c r="S16" s="18"/>
       <c r="T16" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U16" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17">
@@ -2358,32 +2364,32 @@
         <v>16.0</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F17" s="10">
         <v>905.0</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I17" s="13">
         <v>45205.0</v>
       </c>
       <c r="J17" s="17" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K17" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L17" s="10">
         <v>0.0</v>
@@ -2405,10 +2411,10 @@
       </c>
       <c r="S17" s="9"/>
       <c r="T17" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U17" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18">
@@ -2416,32 +2422,32 @@
         <v>17.0</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C18" s="9"/>
       <c r="D18" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F18" s="10">
         <v>806.0</v>
       </c>
       <c r="G18" s="12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H18" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I18" s="13">
         <v>45205.0</v>
       </c>
       <c r="J18" s="17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K18" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L18" s="10">
         <v>0.0</v>
@@ -2463,10 +2469,10 @@
       </c>
       <c r="S18" s="18"/>
       <c r="T18" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U18" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19">
@@ -2474,32 +2480,32 @@
         <v>18.0</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C19" s="9"/>
       <c r="D19" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F19" s="10">
         <v>918.0</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H19" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I19" s="13">
         <v>45205.0</v>
       </c>
       <c r="J19" s="17" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K19" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L19" s="10">
         <v>0.0</v>
@@ -2521,10 +2527,10 @@
       </c>
       <c r="S19" s="18"/>
       <c r="T19" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U19" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20">
@@ -2532,32 +2538,32 @@
         <v>19.0</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C20" s="9"/>
       <c r="D20" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F20" s="10">
         <v>815.0</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H20" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I20" s="13">
         <v>45205.0</v>
       </c>
       <c r="J20" s="17" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K20" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L20" s="10">
         <v>0.0</v>
@@ -2579,10 +2585,10 @@
       </c>
       <c r="S20" s="18"/>
       <c r="T20" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U20" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21">
@@ -2590,32 +2596,32 @@
         <v>20.0</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C21" s="9"/>
       <c r="D21" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F21" s="10">
         <v>894.0</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I21" s="13">
         <v>45205.0</v>
       </c>
       <c r="J21" s="17" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K21" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L21" s="10">
         <v>0.0</v>
@@ -2637,10 +2643,10 @@
       </c>
       <c r="S21" s="18"/>
       <c r="T21" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U21" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22">
@@ -2648,32 +2654,32 @@
         <v>21.0</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C22" s="9"/>
       <c r="D22" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F22" s="10">
         <v>806.0</v>
       </c>
       <c r="G22" s="12" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H22" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I22" s="13">
         <v>45205.0</v>
       </c>
       <c r="J22" s="17" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K22" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L22" s="10">
         <v>0.0</v>
@@ -2695,10 +2701,10 @@
       </c>
       <c r="S22" s="18"/>
       <c r="T22" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U22" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23">
@@ -2706,32 +2712,32 @@
         <v>22.0</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C23" s="9"/>
       <c r="D23" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F23" s="10">
         <v>892.0</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I23" s="13">
         <v>45205.0</v>
       </c>
       <c r="J23" s="17" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="K23" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L23" s="10">
         <v>1.0</v>
@@ -2752,13 +2758,13 @@
         <v>0.0</v>
       </c>
       <c r="S23" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="T23" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U23" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="24">
@@ -2766,32 +2772,32 @@
         <v>23.0</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C24" s="9"/>
       <c r="D24" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F24" s="10">
         <v>811.0</v>
       </c>
       <c r="G24" s="12" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H24" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I24" s="13">
         <v>45205.0</v>
       </c>
       <c r="J24" s="17" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K24" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L24" s="10">
         <v>0.0</v>
@@ -2813,10 +2819,10 @@
       </c>
       <c r="S24" s="18"/>
       <c r="T24" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U24" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="25">
@@ -2824,32 +2830,32 @@
         <v>24.0</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C25" s="9"/>
       <c r="D25" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F25" s="10">
         <v>863.0</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H25" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I25" s="13">
         <v>45207.0</v>
       </c>
       <c r="J25" s="17" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="K25" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L25" s="10">
         <v>0.0</v>
@@ -2871,10 +2877,10 @@
       </c>
       <c r="S25" s="18"/>
       <c r="T25" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U25" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="26">
@@ -2882,32 +2888,32 @@
         <v>25.0</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C26" s="9"/>
       <c r="D26" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F26" s="10">
         <v>790.0</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H26" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I26" s="13">
         <v>45207.0</v>
       </c>
       <c r="J26" s="17" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K26" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L26" s="10">
         <v>0.0</v>
@@ -2929,10 +2935,10 @@
       </c>
       <c r="S26" s="18"/>
       <c r="T26" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U26" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="27" ht="16.5" customHeight="1">
@@ -2940,32 +2946,32 @@
         <v>26.0</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C27" s="9"/>
       <c r="D27" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F27" s="10">
         <v>947.0</v>
       </c>
       <c r="G27" s="23" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H27" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I27" s="13">
         <v>45207.0</v>
       </c>
       <c r="J27" s="17" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K27" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L27" s="10">
         <v>0.0</v>
@@ -2987,10 +2993,10 @@
       </c>
       <c r="S27" s="18"/>
       <c r="T27" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U27" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="28">
@@ -2998,32 +3004,32 @@
         <v>27.0</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C28" s="9"/>
       <c r="D28" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F28" s="10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G28" s="23" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I28" s="13">
         <v>45207.0</v>
       </c>
       <c r="J28" s="17" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K28" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L28" s="10">
         <v>1.0</v>
@@ -3045,10 +3051,10 @@
       </c>
       <c r="S28" s="18"/>
       <c r="T28" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U28" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="29">
@@ -3056,32 +3062,32 @@
         <v>28.0</v>
       </c>
       <c r="B29" s="26" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C29" s="26"/>
       <c r="D29" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G29" s="12" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I29" s="13">
         <v>45208.0</v>
       </c>
       <c r="J29" s="17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K29" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L29" s="10">
         <v>0.0</v>
@@ -3103,10 +3109,10 @@
       </c>
       <c r="S29" s="18"/>
       <c r="T29" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U29" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="30">
@@ -3114,32 +3120,32 @@
         <v>29.0</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C30" s="9"/>
       <c r="D30" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H30" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I30" s="13">
         <v>45208.0</v>
       </c>
       <c r="J30" s="17" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K30" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L30" s="10">
         <v>0.0</v>
@@ -3161,10 +3167,10 @@
       </c>
       <c r="S30" s="18"/>
       <c r="T30" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U30" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="31">
@@ -3172,32 +3178,32 @@
         <v>30.0</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C31" s="9"/>
       <c r="D31" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F31" s="10">
         <v>917.0</v>
       </c>
       <c r="G31" s="23" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H31" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I31" s="13">
         <v>45208.0</v>
       </c>
       <c r="J31" s="17" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K31" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L31" s="10">
         <v>0.0</v>
@@ -3219,10 +3225,10 @@
       </c>
       <c r="S31" s="18"/>
       <c r="T31" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U31" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="32" ht="16.5" customHeight="1">
@@ -3230,32 +3236,32 @@
         <v>31.0</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C32" s="9"/>
       <c r="D32" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F32" s="10">
         <v>877.0</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H32" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I32" s="13">
         <v>45208.0</v>
       </c>
       <c r="J32" s="14" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K32" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L32" s="10">
         <v>1.0</v>
@@ -3277,10 +3283,10 @@
       </c>
       <c r="S32" s="18"/>
       <c r="T32" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U32" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="33">
@@ -3288,32 +3294,32 @@
         <v>32.0</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C33" s="9"/>
       <c r="D33" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F33" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H33" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I33" s="13">
         <v>45208.0</v>
       </c>
       <c r="J33" s="17" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K33" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L33" s="10">
         <v>0.0</v>
@@ -3335,10 +3341,10 @@
       </c>
       <c r="S33" s="18"/>
       <c r="T33" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U33" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="34">
@@ -3346,32 +3352,32 @@
         <v>33.0</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C34" s="9"/>
       <c r="D34" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F34" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G34" s="23" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H34" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I34" s="13">
         <v>45208.0</v>
       </c>
       <c r="J34" s="17" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K34" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L34" s="10">
         <v>0.0</v>
@@ -3393,10 +3399,10 @@
       </c>
       <c r="S34" s="18"/>
       <c r="T34" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U34" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="35">
@@ -3404,32 +3410,32 @@
         <v>34.0</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C35" s="9"/>
       <c r="D35" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F35" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G35" s="23" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H35" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I35" s="13">
         <v>45208.0</v>
       </c>
       <c r="J35" s="17" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="K35" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L35" s="10">
         <v>0.0</v>
@@ -3451,10 +3457,10 @@
       </c>
       <c r="S35" s="18"/>
       <c r="T35" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U35" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="36">
@@ -3462,32 +3468,32 @@
         <v>35.0</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C36" s="9"/>
       <c r="D36" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F36" s="10" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G36" s="12" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H36" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I36" s="13">
         <v>45208.0</v>
       </c>
       <c r="J36" s="17" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K36" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L36" s="10">
         <v>0.0</v>
@@ -3509,10 +3515,10 @@
       </c>
       <c r="S36" s="18"/>
       <c r="T36" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U36" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="37">
@@ -3520,32 +3526,32 @@
         <v>36.0</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C37" s="9"/>
       <c r="D37" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F37" s="10" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G37" s="12" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H37" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I37" s="13">
         <v>45208.0</v>
       </c>
       <c r="J37" s="17" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="K37" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L37" s="10">
         <v>0.0</v>
@@ -3567,10 +3573,10 @@
       </c>
       <c r="S37" s="18"/>
       <c r="T37" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U37" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="38">
@@ -3578,32 +3584,32 @@
         <v>37.0</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C38" s="9"/>
       <c r="D38" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F38" s="10">
         <v>853.0</v>
       </c>
       <c r="G38" s="23" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I38" s="13">
         <v>45208.0</v>
       </c>
       <c r="J38" s="17" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K38" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L38" s="10">
         <v>0.0</v>
@@ -3625,10 +3631,10 @@
       </c>
       <c r="S38" s="18"/>
       <c r="T38" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U38" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="39">
@@ -3636,32 +3642,32 @@
         <v>38.0</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C39" s="9"/>
       <c r="D39" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F39" s="10" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G39" s="12" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I39" s="13">
         <v>45208.0</v>
       </c>
       <c r="J39" s="17" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K39" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L39" s="10">
         <v>0.0</v>
@@ -3683,10 +3689,10 @@
       </c>
       <c r="S39" s="18"/>
       <c r="T39" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U39" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="40">
@@ -3694,32 +3700,32 @@
         <v>39.0</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C40" s="9"/>
       <c r="D40" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F40" s="10">
         <v>882.0</v>
       </c>
       <c r="G40" s="12" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H40" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I40" s="13">
         <v>45208.0</v>
       </c>
       <c r="J40" s="17" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="K40" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="L40" s="10">
         <v>0.0</v>
@@ -3741,10 +3747,10 @@
       </c>
       <c r="S40" s="9"/>
       <c r="T40" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U40" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="41">
@@ -3752,32 +3758,32 @@
         <v>40.0</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C41" s="9"/>
       <c r="D41" s="10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F41" s="10">
         <v>904.0</v>
       </c>
       <c r="G41" s="12" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H41" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I41" s="13">
         <v>45208.0</v>
       </c>
       <c r="J41" s="14" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K41" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L41" s="10">
         <v>0.0</v>
@@ -3798,13 +3804,13 @@
         <v>2.0</v>
       </c>
       <c r="S41" s="9" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="T41" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U41" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="42">
@@ -3812,32 +3818,32 @@
         <v>41.0</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C42" s="9"/>
       <c r="D42" s="10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F42" s="10">
         <v>900.0</v>
       </c>
       <c r="G42" s="12" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H42" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I42" s="13">
         <v>45208.0</v>
       </c>
       <c r="J42" s="17" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K42" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L42" s="10">
         <v>0.0</v>
@@ -3859,7 +3865,7 @@
       </c>
       <c r="S42" s="18"/>
       <c r="U42" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="43">
@@ -3867,32 +3873,32 @@
         <v>42.0</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C43" s="9"/>
       <c r="D43" s="10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F43" s="10">
         <v>855.0</v>
       </c>
       <c r="G43" s="12" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H43" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I43" s="13">
         <v>45208.0</v>
       </c>
       <c r="J43" s="17" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K43" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L43" s="10">
         <v>0.0</v>
@@ -3914,10 +3920,10 @@
       </c>
       <c r="S43" s="18"/>
       <c r="T43" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U43" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="44">
@@ -3925,32 +3931,32 @@
         <v>43.0</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C44" s="9"/>
       <c r="D44" s="10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E44" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F44" s="10">
         <v>844.0</v>
       </c>
       <c r="G44" s="12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H44" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I44" s="13">
         <v>45208.0</v>
       </c>
       <c r="J44" s="17" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K44" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L44" s="10">
         <v>2.0</v>
@@ -3972,10 +3978,10 @@
       </c>
       <c r="S44" s="18"/>
       <c r="T44" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U44" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="45">
@@ -3983,32 +3989,32 @@
         <v>44.0</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C45" s="9"/>
       <c r="D45" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F45" s="10">
         <v>904.0</v>
       </c>
       <c r="G45" s="12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H45" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I45" s="13">
         <v>45208.0</v>
       </c>
       <c r="J45" s="17" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K45" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L45" s="10">
         <v>1.0</v>
@@ -4030,10 +4036,10 @@
       </c>
       <c r="S45" s="18"/>
       <c r="T45" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U45" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="46">
@@ -4041,32 +4047,32 @@
         <v>45.0</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C46" s="9"/>
       <c r="D46" s="10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F46" s="10">
         <v>835.0</v>
       </c>
       <c r="G46" s="12" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="H46" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I46" s="13">
         <v>45208.0</v>
       </c>
       <c r="J46" s="17" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K46" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L46" s="10">
         <v>1.0</v>
@@ -4088,10 +4094,10 @@
       </c>
       <c r="S46" s="18"/>
       <c r="T46" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U46" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="47">
@@ -4099,32 +4105,32 @@
         <v>46.0</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C47" s="9"/>
       <c r="D47" s="10" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F47" s="10">
         <v>892.0</v>
       </c>
       <c r="G47" s="12" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H47" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I47" s="13">
         <v>45208.0</v>
       </c>
       <c r="J47" s="17" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K47" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L47" s="10">
         <v>0.0</v>
@@ -4146,10 +4152,10 @@
       </c>
       <c r="S47" s="18"/>
       <c r="T47" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U47" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="48">
@@ -4157,32 +4163,32 @@
         <v>47.0</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C48" s="9"/>
       <c r="D48" s="10" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F48" s="10">
         <v>894.0</v>
       </c>
       <c r="G48" s="12" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H48" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I48" s="13">
         <v>45208.0</v>
       </c>
       <c r="J48" s="17" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K48" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L48" s="10">
         <v>0.0</v>
@@ -4204,10 +4210,10 @@
       </c>
       <c r="S48" s="18"/>
       <c r="T48" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U48" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="49">
@@ -4215,32 +4221,32 @@
         <v>48.0</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C49" s="9"/>
       <c r="D49" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F49" s="10">
         <v>812.0</v>
       </c>
       <c r="G49" s="12" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="H49" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I49" s="13">
         <v>45208.0</v>
       </c>
       <c r="J49" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K49" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L49" s="10">
         <v>0.0</v>
@@ -4262,10 +4268,10 @@
       </c>
       <c r="S49" s="18"/>
       <c r="T49" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U49" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="50">
@@ -4273,32 +4279,32 @@
         <v>49.0</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C50" s="9"/>
       <c r="D50" s="10" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E50" s="9" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F50" s="10">
         <v>851.0</v>
       </c>
       <c r="G50" s="12" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H50" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I50" s="13">
         <v>45208.0</v>
       </c>
       <c r="J50" s="17" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K50" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L50" s="10">
         <v>0.0</v>
@@ -4319,13 +4325,13 @@
         <v>7.0</v>
       </c>
       <c r="S50" s="9" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="T50" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U50" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="51">
@@ -4333,32 +4339,32 @@
         <v>50.0</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C51" s="9"/>
       <c r="D51" s="10" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F51" s="10">
         <v>864.0</v>
       </c>
       <c r="G51" s="12" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H51" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I51" s="13">
         <v>45208.0</v>
       </c>
       <c r="J51" s="17" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="K51" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L51" s="10">
         <v>0.0</v>
@@ -4380,10 +4386,10 @@
       </c>
       <c r="S51" s="18"/>
       <c r="T51" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U51" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="52">
@@ -4391,32 +4397,32 @@
         <v>51.0</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C52" s="9"/>
       <c r="D52" s="10" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E52" s="9" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F52" s="10" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G52" s="12" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H52" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I52" s="13">
         <v>45209.0</v>
       </c>
       <c r="J52" s="17" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K52" s="10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="L52" s="10">
         <v>1.0</v>
@@ -4438,10 +4444,10 @@
       </c>
       <c r="S52" s="18"/>
       <c r="T52" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U52" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="53">
@@ -4449,32 +4455,32 @@
         <v>52.0</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C53" s="9"/>
       <c r="D53" s="10" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F53" s="10">
         <v>875.0</v>
       </c>
       <c r="G53" s="12" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H53" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I53" s="13">
         <v>45209.0</v>
       </c>
       <c r="J53" s="17" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="K53" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L53" s="10">
         <v>0.0</v>
@@ -4496,10 +4502,10 @@
       </c>
       <c r="S53" s="18"/>
       <c r="T53" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U53" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="54">
@@ -4507,32 +4513,32 @@
         <v>53.0</v>
       </c>
       <c r="B54" s="27" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C54" s="27"/>
       <c r="D54" s="10" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E54" s="9" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F54" s="10">
         <v>867.0</v>
       </c>
       <c r="G54" s="12" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H54" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I54" s="13">
         <v>45209.0</v>
       </c>
       <c r="J54" s="17" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K54" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L54" s="10">
         <v>0.0</v>
@@ -4554,10 +4560,10 @@
       </c>
       <c r="S54" s="18"/>
       <c r="T54" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U54" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="55">
@@ -4565,32 +4571,32 @@
         <v>54.0</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C55" s="9"/>
       <c r="D55" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F55" s="10">
         <v>830.0</v>
       </c>
       <c r="G55" s="12" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H55" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I55" s="13">
         <v>45209.0</v>
       </c>
       <c r="J55" s="17" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="K55" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L55" s="10">
         <v>0.0</v>
@@ -4612,10 +4618,10 @@
       </c>
       <c r="S55" s="18"/>
       <c r="T55" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U55" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="56">
@@ -4623,32 +4629,32 @@
         <v>55.0</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C56" s="9"/>
       <c r="D56" s="10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E56" s="9" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F56" s="10">
         <v>852.0</v>
       </c>
       <c r="G56" s="12" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H56" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I56" s="13">
         <v>45209.0</v>
       </c>
       <c r="J56" s="17" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K56" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L56" s="10">
         <v>1.0</v>
@@ -4670,10 +4676,10 @@
       </c>
       <c r="S56" s="18"/>
       <c r="T56" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U56" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="57">
@@ -4681,32 +4687,32 @@
         <v>56.0</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C57" s="9"/>
       <c r="D57" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F57" s="10">
         <v>859.0</v>
       </c>
       <c r="G57" s="12" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="H57" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I57" s="13">
         <v>45209.0</v>
       </c>
       <c r="J57" s="17" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K57" s="28" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L57" s="10">
         <v>0.0</v>
@@ -4728,10 +4734,10 @@
       </c>
       <c r="S57" s="18"/>
       <c r="T57" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U57" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="58">
@@ -4739,32 +4745,32 @@
         <v>57.0</v>
       </c>
       <c r="B58" s="9" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C58" s="9"/>
       <c r="D58" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E58" s="9" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F58" s="10">
         <v>916.0</v>
       </c>
       <c r="G58" s="12" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H58" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I58" s="13">
         <v>45209.0</v>
       </c>
       <c r="J58" s="17" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="K58" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L58" s="10">
         <v>0.0</v>
@@ -4786,10 +4792,10 @@
       </c>
       <c r="S58" s="18"/>
       <c r="T58" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U58" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="59">
@@ -4797,32 +4803,32 @@
         <v>58.0</v>
       </c>
       <c r="B59" s="9" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C59" s="9"/>
       <c r="D59" s="10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F59" s="10">
         <v>881.0</v>
       </c>
       <c r="G59" s="12" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="H59" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I59" s="13">
         <v>45209.0</v>
       </c>
       <c r="J59" s="17" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="K59" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L59" s="10">
         <v>0.0</v>
@@ -4844,10 +4850,10 @@
       </c>
       <c r="S59" s="18"/>
       <c r="T59" s="19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U59" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="60">
@@ -4855,32 +4861,32 @@
         <v>59.0</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C60" s="18"/>
       <c r="D60" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E60" s="9" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F60" s="10">
         <v>1073.0</v>
       </c>
       <c r="G60" s="12" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="H60" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I60" s="13">
         <v>45216.0</v>
       </c>
       <c r="J60" s="17" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="K60" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L60" s="10">
         <v>0.0</v>
@@ -4901,13 +4907,13 @@
         <v>0.0</v>
       </c>
       <c r="S60" s="9" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="T60" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U60" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="61">
@@ -4915,32 +4921,32 @@
         <v>60.0</v>
       </c>
       <c r="B61" s="9" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C61" s="18"/>
       <c r="D61" s="10" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F61" s="10">
         <v>1062.0</v>
       </c>
       <c r="G61" s="12" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="H61" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I61" s="13">
         <v>45216.0</v>
       </c>
       <c r="J61" s="14" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="K61" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L61" s="10">
         <v>0.0</v>
@@ -4962,10 +4968,10 @@
       </c>
       <c r="S61" s="18"/>
       <c r="T61" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U61" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="62">
@@ -4973,32 +4979,32 @@
         <v>61.0</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C62" s="18"/>
       <c r="D62" s="10" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E62" s="9" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F62" s="10">
         <v>958.0</v>
       </c>
       <c r="G62" s="12" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="H62" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I62" s="13">
         <v>45216.0</v>
       </c>
       <c r="J62" s="17" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="K62" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L62" s="10">
         <v>0.0</v>
@@ -5019,13 +5025,13 @@
         <v>0.0</v>
       </c>
       <c r="S62" s="9" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="T62" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U62" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="63">
@@ -5033,32 +5039,32 @@
         <v>62.0</v>
       </c>
       <c r="B63" s="9" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C63" s="18"/>
       <c r="D63" s="10" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E63" s="9" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F63" s="29">
         <v>898.0</v>
       </c>
       <c r="G63" s="12" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="H63" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I63" s="13">
         <v>45216.0</v>
       </c>
       <c r="J63" s="17" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="K63" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L63" s="10">
         <v>0.0</v>
@@ -5079,13 +5085,13 @@
         <v>0.0</v>
       </c>
       <c r="S63" s="9" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="T63" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U63" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="64">
@@ -5093,32 +5099,32 @@
         <v>63.0</v>
       </c>
       <c r="B64" s="9" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C64" s="18"/>
       <c r="D64" s="10" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E64" s="9" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F64" s="10">
         <v>947.0</v>
       </c>
       <c r="G64" s="12" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="H64" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I64" s="13">
         <v>45216.0</v>
       </c>
       <c r="J64" s="17" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="K64" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L64" s="10">
         <v>1.0</v>
@@ -5139,13 +5145,13 @@
         <v>0.0</v>
       </c>
       <c r="S64" s="9" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="T64" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U64" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="65">
@@ -5153,32 +5159,32 @@
         <v>64.0</v>
       </c>
       <c r="B65" s="9" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C65" s="18"/>
       <c r="D65" s="10" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E65" s="9" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F65" s="10">
         <v>1093.0</v>
       </c>
       <c r="G65" s="12" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="H65" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I65" s="13">
         <v>45216.0</v>
       </c>
       <c r="J65" s="14" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="K65" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L65" s="10">
         <v>5.0</v>
@@ -5199,13 +5205,13 @@
         <v>0.0</v>
       </c>
       <c r="S65" s="9" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="T65" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U65" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="66">
@@ -5213,32 +5219,32 @@
         <v>65.0</v>
       </c>
       <c r="B66" s="9" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C66" s="18"/>
       <c r="D66" s="10" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E66" s="9" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F66" s="10">
         <v>939.0</v>
       </c>
       <c r="G66" s="12" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="H66" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I66" s="13">
         <v>45216.0</v>
       </c>
       <c r="J66" s="17" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="K66" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L66" s="10">
         <v>0.0</v>
@@ -5259,13 +5265,13 @@
         <v>1.0</v>
       </c>
       <c r="S66" s="9" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="T66" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U66" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="67">
@@ -5273,32 +5279,32 @@
         <v>66.0</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C67" s="18"/>
       <c r="D67" s="10" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F67" s="10">
         <v>863.0</v>
       </c>
       <c r="G67" s="12" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="H67" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I67" s="13">
         <v>45216.0</v>
       </c>
       <c r="J67" s="17" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="K67" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L67" s="10">
         <v>0.0</v>
@@ -5319,13 +5325,13 @@
         <v>4.0</v>
       </c>
       <c r="S67" s="9" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="T67" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U67" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="68">
@@ -5333,32 +5339,32 @@
         <v>67.0</v>
       </c>
       <c r="B68" s="9" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C68" s="18"/>
       <c r="D68" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E68" s="9" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F68" s="10">
         <v>801.0</v>
       </c>
       <c r="G68" s="12" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="H68" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I68" s="13">
         <v>45216.0</v>
       </c>
       <c r="J68" s="17" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="K68" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L68" s="10">
         <v>0.0</v>
@@ -5379,13 +5385,13 @@
         <v>0.0</v>
       </c>
       <c r="S68" s="9" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="T68" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U68" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="69">
@@ -5393,32 +5399,32 @@
         <v>68.0</v>
       </c>
       <c r="B69" s="9" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C69" s="18"/>
       <c r="D69" s="10" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E69" s="9" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F69" s="10">
         <v>1001.0</v>
       </c>
       <c r="G69" s="12" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="H69" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I69" s="13">
         <v>45216.0</v>
       </c>
       <c r="J69" s="17" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="K69" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L69" s="10">
         <v>4.0</v>
@@ -5439,13 +5445,13 @@
         <v>0.0</v>
       </c>
       <c r="S69" s="9" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="T69" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U69" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="70">
@@ -5453,32 +5459,32 @@
         <v>69.0</v>
       </c>
       <c r="B70" s="9" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C70" s="18"/>
       <c r="D70" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E70" s="9" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F70" s="10">
         <v>946.0</v>
       </c>
       <c r="G70" s="12" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="H70" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I70" s="13">
         <v>45216.0</v>
       </c>
       <c r="J70" s="17" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="K70" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L70" s="10">
         <v>1.0</v>
@@ -5499,13 +5505,13 @@
         <v>0.0</v>
       </c>
       <c r="S70" s="9" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="T70" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U70" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="71">
@@ -5513,32 +5519,32 @@
         <v>70.0</v>
       </c>
       <c r="B71" s="9" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C71" s="18"/>
       <c r="D71" s="10" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E71" s="9" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F71" s="10">
         <v>884.0</v>
       </c>
       <c r="G71" s="12" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="H71" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I71" s="13">
         <v>45216.0</v>
       </c>
       <c r="J71" s="17" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="K71" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L71" s="10">
         <v>1.0</v>
@@ -5559,13 +5565,13 @@
         <v>0.0</v>
       </c>
       <c r="S71" s="9" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="T71" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U71" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="72">
@@ -5573,32 +5579,32 @@
         <v>71.0</v>
       </c>
       <c r="B72" s="9" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C72" s="18"/>
       <c r="D72" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E72" s="9" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F72" s="10">
         <v>899.0</v>
       </c>
       <c r="G72" s="12" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="H72" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I72" s="13">
         <v>45216.0</v>
       </c>
       <c r="J72" s="17" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="K72" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L72" s="10">
         <v>0.0</v>
@@ -5619,13 +5625,13 @@
         <v>0.0</v>
       </c>
       <c r="S72" s="9" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="T72" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U72" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="73">
@@ -5633,32 +5639,32 @@
         <v>72.0</v>
       </c>
       <c r="B73" s="9" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C73" s="18"/>
       <c r="D73" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E73" s="9" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F73" s="10" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="G73" s="12" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="H73" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I73" s="13">
         <v>45221.0</v>
       </c>
       <c r="J73" s="17" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="K73" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L73" s="10">
         <v>0.0</v>
@@ -5680,7 +5686,7 @@
       </c>
       <c r="S73" s="18"/>
       <c r="T73" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="74">
@@ -5688,32 +5694,32 @@
         <v>73.0</v>
       </c>
       <c r="B74" s="9" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C74" s="18"/>
       <c r="D74" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E74" s="9" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="F74" s="10">
         <v>882.0</v>
       </c>
       <c r="G74" s="12" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="H74" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I74" s="13">
         <v>45221.0</v>
       </c>
       <c r="J74" s="17" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="K74" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L74" s="10">
         <v>0.0</v>
@@ -5734,13 +5740,13 @@
         <v>1.0</v>
       </c>
       <c r="S74" s="9" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="T74" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U74" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="75">
@@ -5748,32 +5754,32 @@
         <v>74.0</v>
       </c>
       <c r="B75" s="9" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C75" s="18"/>
       <c r="D75" s="10" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="F75" s="10">
         <v>928.0</v>
       </c>
       <c r="G75" s="12" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="H75" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I75" s="13">
         <v>45221.0</v>
       </c>
       <c r="J75" s="17" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="K75" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L75" s="10">
         <v>1.0</v>
@@ -5794,13 +5800,13 @@
         <v>0.0</v>
       </c>
       <c r="S75" s="9" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="T75" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U75" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="76">
@@ -5808,32 +5814,32 @@
         <v>75.0</v>
       </c>
       <c r="B76" s="9" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C76" s="18"/>
       <c r="D76" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E76" s="9" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="F76" s="10">
         <v>864.0</v>
       </c>
       <c r="G76" s="12" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="H76" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I76" s="13">
         <v>45221.0</v>
       </c>
       <c r="J76" s="17" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="K76" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L76" s="10">
         <v>0.0</v>
@@ -5854,13 +5860,13 @@
         <v>0.0</v>
       </c>
       <c r="S76" s="9" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="T76" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U76" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="77">
@@ -5868,32 +5874,32 @@
         <v>76.0</v>
       </c>
       <c r="B77" s="9" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C77" s="18"/>
       <c r="D77" s="10" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E77" s="9" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F77" s="10">
         <v>879.0</v>
       </c>
       <c r="G77" s="12" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="H77" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I77" s="13">
         <v>45221.0</v>
       </c>
       <c r="J77" s="14" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K77" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L77" s="10">
         <v>2.0</v>
@@ -5914,13 +5920,13 @@
         <v>1.0</v>
       </c>
       <c r="S77" s="9" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="T77" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="U77" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="78">
@@ -5928,102 +5934,165 @@
         <v>77.0</v>
       </c>
       <c r="B78" s="9" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C78" s="18"/>
       <c r="D78" s="10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E78" s="9" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F78" s="10">
         <v>815.0</v>
       </c>
       <c r="G78" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="H78" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I78" s="13">
         <v>45222.0</v>
       </c>
       <c r="J78" s="12" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="K78" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
+      </c>
+      <c r="L78" s="10">
+        <v>3.0</v>
+      </c>
+      <c r="M78" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="N78" s="10">
+        <v>1.0</v>
+      </c>
+      <c r="O78" s="10">
+        <v>5.0</v>
+      </c>
+      <c r="P78" s="10">
+        <v>1.0</v>
+      </c>
+      <c r="Q78" s="10">
+        <v>3.0</v>
       </c>
       <c r="S78" s="18"/>
+      <c r="U78" s="10" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="10">
         <v>78.0</v>
       </c>
       <c r="B79" s="9" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C79" s="18"/>
       <c r="D79" s="10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E79" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="F79" s="10">
         <v>908.0</v>
       </c>
       <c r="G79" s="12" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="H79" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I79" s="13">
         <v>45222.0</v>
       </c>
       <c r="J79" s="12" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="K79" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
+      </c>
+      <c r="L79" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="M79" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="N79" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="O79" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="P79" s="10">
+        <v>3.0</v>
+      </c>
+      <c r="Q79" s="10">
+        <v>3.0</v>
       </c>
       <c r="S79" s="18"/>
+      <c r="U79" s="10" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="10">
         <v>79.0</v>
       </c>
       <c r="B80" s="9" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C80" s="18"/>
       <c r="D80" s="10" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E80" s="9" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="F80" s="10">
         <v>879.0</v>
       </c>
       <c r="G80" s="12" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="H80" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I80" s="13">
         <v>45222.0</v>
       </c>
       <c r="J80" s="12" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="K80" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
+      </c>
+      <c r="L80" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="M80" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="N80" s="10">
+        <v>0.0</v>
+      </c>
+      <c r="O80" s="10">
+        <v>2.0</v>
+      </c>
+      <c r="P80" s="10">
+        <v>1.0</v>
+      </c>
+      <c r="Q80" s="10">
+        <v>2.0</v>
       </c>
       <c r="S80" s="18"/>
+      <c r="U80" s="10" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="81">
       <c r="B81" s="18"/>

</xml_diff>